<commit_message>
update SA GA and fine-tuning code
</commit_message>
<xml_diff>
--- a/data/data-23-24-2.xlsx
+++ b/data/data-23-24-2.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17700"/>
+    <workbookView windowWidth="22185" windowHeight="9060" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="classRoomLT" sheetId="9" r:id="rId1"/>
@@ -12,7 +12,6 @@
     <sheet name="registrationClass" sheetId="3" r:id="rId3"/>
     <sheet name="subject" sheetId="4" r:id="rId4"/>
     <sheet name="date" sheetId="5" r:id="rId5"/>
-    <sheet name="academyYear" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -32,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="136">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="127">
   <si>
     <t>ID</t>
   </si>
@@ -40,18 +39,9 @@
     <t>Classroom name</t>
   </si>
   <si>
-    <t>Real capacity</t>
-  </si>
-  <si>
     <t>Exam capacity</t>
   </si>
   <si>
-    <t>Classroom type</t>
-  </si>
-  <si>
-    <t>Building Id</t>
-  </si>
-  <si>
     <t>RD405</t>
   </si>
   <si>
@@ -91,18 +81,12 @@
     <t>Subject name</t>
   </si>
   <si>
-    <t>Estimate class size</t>
-  </si>
-  <si>
     <t>Real class size</t>
   </si>
   <si>
     <t>Grade name</t>
   </si>
   <si>
-    <t>Semester id</t>
-  </si>
-  <si>
     <t>214231-01</t>
   </si>
   <si>
@@ -319,18 +303,12 @@
     <t>Subject id</t>
   </si>
   <si>
-    <t>Credit</t>
-  </si>
-  <si>
     <t>Type</t>
   </si>
   <si>
     <t>Exam time</t>
   </si>
   <si>
-    <t>Lesson time</t>
-  </si>
-  <si>
     <t>214231</t>
   </si>
   <si>
@@ -434,12 +412,6 @@
   </si>
   <si>
     <t>2024-06-20</t>
-  </si>
-  <si>
-    <t>Academy year</t>
-  </si>
-  <si>
-    <t>semester</t>
   </si>
 </sst>
 </file>
@@ -1067,17 +1039,17 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1">
@@ -1105,10 +1077,6 @@
     <xf numFmtId="178" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1642,10 +1610,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="5"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="2"/>
+  <cols>
+    <col min="3" max="3" width="14.2857142857143" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1655,114 +1626,60 @@
       <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+    </row>
+    <row r="2" spans="1:3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C2">
-        <v>80</v>
-      </c>
-      <c r="D2">
         <v>40</v>
       </c>
-      <c r="E2">
-        <v>0</v>
-      </c>
-      <c r="F2">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>100</v>
-      </c>
-      <c r="D3">
         <v>50</v>
       </c>
-      <c r="E3">
-        <v>0</v>
-      </c>
-      <c r="F3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C4">
-        <v>80</v>
-      </c>
-      <c r="D4">
         <v>40</v>
       </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5">
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C5">
-        <v>80</v>
-      </c>
-      <c r="D5">
         <v>40</v>
       </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+    </row>
+    <row r="6" spans="1:3">
       <c r="A6">
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="C6">
-        <v>80</v>
-      </c>
-      <c r="D6">
         <v>40</v>
-      </c>
-      <c r="E6">
-        <v>0</v>
-      </c>
-      <c r="F6">
-        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1774,127 +1691,73 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F6"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="5"/>
+  <dimension ref="A1:C6"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="5" outlineLevelCol="2"/>
   <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:3">
+      <c r="A1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="3">
+        <v>4</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" s="3">
+        <v>5</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" s="3">
+        <v>6</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
-      <c r="A2" s="1">
-        <v>4</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="C4" s="3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" s="3">
+        <v>7</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C5" s="3">
         <v>40</v>
       </c>
-      <c r="D2" s="1">
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" s="3">
+        <v>8</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" s="3">
         <v>40</v>
-      </c>
-      <c r="E2" s="1">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="1">
-        <v>5</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="1">
-        <v>40</v>
-      </c>
-      <c r="D3" s="1">
-        <v>40</v>
-      </c>
-      <c r="E3" s="1">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="1">
-        <v>6</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="1">
-        <v>40</v>
-      </c>
-      <c r="D4" s="1">
-        <v>40</v>
-      </c>
-      <c r="E4" s="1">
-        <v>1</v>
-      </c>
-      <c r="F4" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="1">
-        <v>7</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C5" s="1">
-        <v>40</v>
-      </c>
-      <c r="D5" s="1">
-        <v>40</v>
-      </c>
-      <c r="E5" s="1">
-        <v>1</v>
-      </c>
-      <c r="F5" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="1">
-        <v>8</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6" s="1">
-        <v>40</v>
-      </c>
-      <c r="D6" s="1">
-        <v>40</v>
-      </c>
-      <c r="E6" s="1">
-        <v>1</v>
-      </c>
-      <c r="F6" s="1">
-        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -1906,1148 +1769,701 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H52"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="7"/>
+  <dimension ref="A1:E49"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="4"/>
   <cols>
     <col min="1" max="1" width="13.5714285714286" style="10" customWidth="1"/>
     <col min="2" max="2" width="37" style="10" customWidth="1"/>
-    <col min="3" max="3" width="18.7142857142857" style="10" customWidth="1"/>
-    <col min="4" max="4" width="14.2857142857143" style="10" customWidth="1"/>
-    <col min="5" max="5" width="12.5714285714286" customWidth="1"/>
-    <col min="6" max="6" width="10.4285714285714" customWidth="1"/>
-    <col min="7" max="7" width="12.4285714285714" customWidth="1"/>
+    <col min="3" max="3" width="14.2857142857143" style="10" customWidth="1"/>
+    <col min="4" max="4" width="12.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:8">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="3" customFormat="1" spans="1:5">
+      <c r="A1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="E1" s="11"/>
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="B2" s="9" t="s">
         <v>19</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H1" s="11"/>
-    </row>
-    <row r="2" spans="1:7">
-      <c r="A2" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B2" s="9" t="s">
-        <v>24</v>
       </c>
       <c r="C2" s="12">
         <v>110</v>
       </c>
-      <c r="D2" s="12">
-        <v>110</v>
-      </c>
-      <c r="E2" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="13">
-        <v>1</v>
-      </c>
-      <c r="G2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+      <c r="D2" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C3" s="12">
         <v>109</v>
       </c>
-      <c r="D3" s="12">
-        <v>109</v>
-      </c>
-      <c r="E3" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="13">
-        <v>2</v>
-      </c>
-      <c r="G3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7">
+      <c r="D3" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C4" s="12">
         <v>150</v>
       </c>
-      <c r="D4" s="12">
-        <v>150</v>
-      </c>
-      <c r="E4" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="13">
-        <v>3</v>
-      </c>
-      <c r="G4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7">
+      <c r="D4" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
       <c r="A5" s="9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C5" s="12">
         <v>110</v>
       </c>
-      <c r="D5" s="12">
-        <v>110</v>
-      </c>
-      <c r="E5" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F5" s="13">
-        <v>4</v>
-      </c>
-      <c r="G5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7">
+      <c r="D5" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
       <c r="A6" s="9" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C6" s="12">
         <v>60</v>
       </c>
-      <c r="D6" s="12">
-        <v>60</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F6" s="13">
-        <v>5</v>
-      </c>
-      <c r="G6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7">
+      <c r="D6" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
       <c r="A7" s="9" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C7" s="12">
         <v>122</v>
       </c>
-      <c r="D7" s="12">
-        <v>122</v>
-      </c>
-      <c r="E7" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F7" s="13">
-        <v>6</v>
-      </c>
-      <c r="G7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7">
+      <c r="D7" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
       <c r="A8" s="9" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C8" s="12">
         <v>60</v>
       </c>
-      <c r="D8" s="12">
-        <v>60</v>
-      </c>
-      <c r="E8" s="9" t="s">
+      <c r="D8" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="F8" s="13">
-        <v>7</v>
-      </c>
-      <c r="G8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7">
-      <c r="A9" s="9" t="s">
-        <v>35</v>
-      </c>
       <c r="B9" s="9" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C9" s="12">
         <v>111</v>
       </c>
-      <c r="D9" s="12">
-        <v>111</v>
-      </c>
-      <c r="E9" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="13">
-        <v>8</v>
-      </c>
-      <c r="G9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7">
+      <c r="D9" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4">
       <c r="A10" s="9" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C10" s="12">
         <v>112</v>
       </c>
-      <c r="D10" s="12">
-        <v>112</v>
-      </c>
-      <c r="E10" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F10" s="13">
-        <v>9</v>
-      </c>
-      <c r="G10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7">
+      <c r="D10" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4">
       <c r="A11" s="9" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C11" s="12">
         <v>112</v>
       </c>
-      <c r="D11" s="12">
-        <v>112</v>
-      </c>
-      <c r="E11" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F11" s="13">
-        <v>10</v>
-      </c>
-      <c r="G11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7">
+      <c r="D11" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4">
       <c r="A12" s="9" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C12" s="12">
         <v>120</v>
       </c>
-      <c r="D12" s="12">
-        <v>120</v>
-      </c>
-      <c r="E12" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="13">
-        <v>11</v>
-      </c>
-      <c r="G12">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7">
+      <c r="D12" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4">
       <c r="A13" s="9" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="C13" s="12">
         <v>121</v>
       </c>
-      <c r="D13" s="12">
-        <v>121</v>
-      </c>
-      <c r="E13" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F13" s="13">
-        <v>12</v>
-      </c>
-      <c r="G13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7">
+      <c r="D13" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
       <c r="A14" s="9" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C14" s="12">
         <v>110</v>
       </c>
-      <c r="D14" s="12">
-        <v>110</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F14" s="13">
-        <v>13</v>
-      </c>
-      <c r="G14">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7">
+      <c r="D14" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4">
       <c r="A15" s="9" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C15" s="12">
         <v>114</v>
       </c>
-      <c r="D15" s="12">
-        <v>114</v>
-      </c>
-      <c r="E15" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F15" s="13">
-        <v>14</v>
-      </c>
-      <c r="G15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7">
+      <c r="D15" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="9" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="C16" s="12">
         <v>152</v>
       </c>
-      <c r="D16" s="12">
-        <v>152</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F16" s="13">
-        <v>15</v>
-      </c>
-      <c r="G16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7">
+      <c r="D16" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="9" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C17" s="12">
         <v>101</v>
       </c>
-      <c r="D17" s="12">
-        <v>101</v>
-      </c>
-      <c r="E17" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F17" s="13">
-        <v>16</v>
-      </c>
-      <c r="G17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7">
+      <c r="D17" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="9" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C18" s="12">
         <v>30</v>
       </c>
-      <c r="D18" s="12">
-        <v>30</v>
-      </c>
-      <c r="E18" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F18" s="13">
-        <v>17</v>
-      </c>
-      <c r="G18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7">
+      <c r="D18" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4">
       <c r="A19" s="9" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C19" s="12">
         <v>100</v>
       </c>
-      <c r="D19" s="12">
-        <v>100</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F19" s="13">
-        <v>18</v>
-      </c>
-      <c r="G19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7">
+      <c r="D19" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4">
       <c r="A20" s="9" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C20" s="12">
         <v>100</v>
       </c>
-      <c r="D20" s="12">
-        <v>100</v>
-      </c>
-      <c r="E20" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F20" s="13">
-        <v>19</v>
-      </c>
-      <c r="G20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:7">
+      <c r="D20" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="9" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C21" s="12">
         <v>109</v>
       </c>
-      <c r="D21" s="12">
-        <v>109</v>
-      </c>
-      <c r="E21" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F21" s="13">
-        <v>20</v>
-      </c>
-      <c r="G21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:7">
+      <c r="D21" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4">
       <c r="A22" s="9" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C22" s="12">
         <v>102</v>
       </c>
-      <c r="D22" s="12">
-        <v>102</v>
-      </c>
-      <c r="E22" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F22" s="13">
-        <v>21</v>
-      </c>
-      <c r="G22">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23" spans="1:7">
+      <c r="D22" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
       <c r="A23" s="9" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C23" s="12">
         <v>93</v>
       </c>
-      <c r="D23" s="12">
-        <v>93</v>
-      </c>
-      <c r="E23" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F23" s="13">
-        <v>22</v>
-      </c>
-      <c r="G23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:7">
+      <c r="D23" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
       <c r="A24" s="9" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C24" s="12">
         <v>111</v>
       </c>
-      <c r="D24" s="12">
-        <v>111</v>
-      </c>
-      <c r="E24" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F24" s="13">
-        <v>23</v>
-      </c>
-      <c r="G24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:7">
+      <c r="D24" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
       <c r="A25" s="9" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C25" s="12">
         <v>113</v>
       </c>
-      <c r="D25" s="12">
-        <v>113</v>
-      </c>
-      <c r="E25" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F25" s="13">
-        <v>24</v>
-      </c>
-      <c r="G25">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7">
+      <c r="D25" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
       <c r="A26" s="9" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C26" s="12">
         <v>114</v>
       </c>
-      <c r="D26" s="12">
-        <v>114</v>
-      </c>
-      <c r="E26" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F26" s="13">
-        <v>25</v>
-      </c>
-      <c r="G26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:7">
+      <c r="D26" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
       <c r="A27" s="9" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C27" s="12">
         <v>111</v>
       </c>
-      <c r="D27" s="12">
-        <v>111</v>
-      </c>
-      <c r="E27" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F27" s="13">
-        <v>26</v>
-      </c>
-      <c r="G27">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7">
+      <c r="D27" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
       <c r="A28" s="9" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C28" s="12">
         <v>111</v>
       </c>
-      <c r="D28" s="12">
-        <v>111</v>
-      </c>
-      <c r="E28" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F28" s="13">
-        <v>27</v>
-      </c>
-      <c r="G28">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7">
+      <c r="D28" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
       <c r="A29" s="9" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C29" s="12">
         <v>97</v>
       </c>
-      <c r="D29" s="12">
-        <v>97</v>
-      </c>
-      <c r="E29" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F29" s="13">
-        <v>28</v>
-      </c>
-      <c r="G29">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7">
+      <c r="D29" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
       <c r="A30" s="9" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C30" s="12">
         <v>114</v>
       </c>
-      <c r="D30" s="12">
-        <v>114</v>
-      </c>
-      <c r="E30" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F30" s="13">
-        <v>29</v>
-      </c>
-      <c r="G30">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7">
+      <c r="D30" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
       <c r="A31" s="9" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C31" s="12">
         <v>111</v>
       </c>
-      <c r="D31" s="12">
-        <v>111</v>
-      </c>
-      <c r="E31" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F31" s="13">
-        <v>30</v>
-      </c>
-      <c r="G31">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7">
+      <c r="D31" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4">
       <c r="A32" s="9" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C32" s="12">
         <v>72</v>
       </c>
-      <c r="D32" s="12">
-        <v>72</v>
-      </c>
-      <c r="E32" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F32" s="13">
-        <v>31</v>
-      </c>
-      <c r="G32">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="33" spans="1:7">
+      <c r="D32" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4">
       <c r="A33" s="9" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C33" s="12">
         <v>73</v>
       </c>
-      <c r="D33" s="12">
-        <v>73</v>
-      </c>
-      <c r="E33" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F33" s="13">
-        <v>32</v>
-      </c>
-      <c r="G33">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7">
+      <c r="D33" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4">
       <c r="A34" s="9" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C34" s="12">
         <v>100</v>
       </c>
-      <c r="D34" s="12">
-        <v>100</v>
-      </c>
-      <c r="E34" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F34" s="13">
-        <v>33</v>
-      </c>
-      <c r="G34">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7">
+      <c r="D34" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4">
       <c r="A35" s="9" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C35" s="12">
         <v>99</v>
       </c>
-      <c r="D35" s="12">
-        <v>99</v>
-      </c>
-      <c r="E35" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F35" s="13">
-        <v>34</v>
-      </c>
-      <c r="G35">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7">
+      <c r="D35" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4">
       <c r="A36" s="9" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C36" s="12">
         <v>110</v>
       </c>
-      <c r="D36" s="12">
-        <v>110</v>
-      </c>
-      <c r="E36" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F36" s="13">
-        <v>35</v>
-      </c>
-      <c r="G36">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="37" spans="1:7">
+      <c r="D36" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4">
       <c r="A37" s="9" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C37" s="12">
         <v>110</v>
       </c>
-      <c r="D37" s="12">
-        <v>110</v>
-      </c>
-      <c r="E37" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F37" s="13">
-        <v>36</v>
-      </c>
-      <c r="G37">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="38" spans="1:7">
+      <c r="D37" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4">
       <c r="A38" s="9" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C38" s="12">
         <v>150</v>
       </c>
-      <c r="D38" s="12">
-        <v>150</v>
-      </c>
-      <c r="E38" s="9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F38" s="13">
-        <v>37</v>
-      </c>
-      <c r="G38">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7">
+      <c r="D38" s="9" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4">
       <c r="A39" s="9" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C39" s="12">
         <v>97</v>
       </c>
-      <c r="D39" s="12">
-        <v>97</v>
-      </c>
-      <c r="E39" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F39" s="13">
-        <v>38</v>
-      </c>
-      <c r="G39">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7">
+      <c r="D39" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4">
       <c r="A40" s="9" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C40" s="12">
         <v>62</v>
       </c>
-      <c r="D40" s="12">
-        <v>62</v>
-      </c>
-      <c r="E40" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F40" s="13">
-        <v>39</v>
-      </c>
-      <c r="G40">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="41" spans="1:7">
+      <c r="D40" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4">
       <c r="A41" s="9" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C41" s="12">
         <v>92</v>
       </c>
-      <c r="D41" s="12">
-        <v>92</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F41" s="13">
-        <v>40</v>
-      </c>
-      <c r="G41">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="42" spans="1:7">
+      <c r="D41" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4">
       <c r="A42" s="9" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C42" s="12">
         <v>76</v>
       </c>
-      <c r="D42" s="12">
-        <v>76</v>
-      </c>
-      <c r="E42" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F42" s="13">
-        <v>41</v>
-      </c>
-      <c r="G42">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="43" spans="1:7">
+      <c r="D42" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4">
       <c r="A43" s="9" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C43" s="12">
         <v>31</v>
       </c>
-      <c r="D43" s="12">
-        <v>31</v>
-      </c>
-      <c r="E43" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F43" s="13">
-        <v>42</v>
-      </c>
-      <c r="G43">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7">
+      <c r="D43" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4">
       <c r="A44" s="9" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C44" s="12">
         <v>112</v>
       </c>
-      <c r="D44" s="12">
-        <v>112</v>
-      </c>
-      <c r="E44" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F44" s="13">
-        <v>43</v>
-      </c>
-      <c r="G44">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7">
+      <c r="D44" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4">
       <c r="A45" s="9" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C45" s="12">
         <v>116</v>
       </c>
-      <c r="D45" s="12">
-        <v>116</v>
-      </c>
-      <c r="E45" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F45" s="13">
-        <v>44</v>
-      </c>
-      <c r="G45">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7">
+      <c r="D45" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4">
       <c r="A46" s="9" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C46" s="12">
         <v>114</v>
       </c>
-      <c r="D46" s="12">
-        <v>114</v>
-      </c>
-      <c r="E46" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="F46" s="13">
-        <v>45</v>
-      </c>
-      <c r="G46">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7">
+      <c r="D46" s="9" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4">
       <c r="A47" s="9" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C47" s="12">
         <v>153</v>
       </c>
-      <c r="D47" s="12">
-        <v>153</v>
-      </c>
-      <c r="E47" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F47" s="13">
-        <v>46</v>
-      </c>
-      <c r="G47">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7">
+      <c r="D47" s="9" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4">
       <c r="A48" s="9" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C48" s="12">
         <v>110</v>
       </c>
-      <c r="D48" s="12">
-        <v>110</v>
-      </c>
-      <c r="E48" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F48" s="13">
-        <v>47</v>
-      </c>
-      <c r="G48">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="49" spans="1:7">
+      <c r="D48" s="9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4">
       <c r="A49" s="9" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C49" s="12">
         <v>111</v>
       </c>
-      <c r="D49" s="12">
-        <v>111</v>
-      </c>
-      <c r="E49" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="F49" s="13">
-        <v>48</v>
-      </c>
-      <c r="G49">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="52" spans="3:3">
-      <c r="C52" s="14"/>
+      <c r="D49" s="9" t="s">
+        <v>25</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3058,513 +2474,362 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:F25"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="5"/>
+  <dimension ref="A1:D25"/>
+  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelCol="3"/>
   <cols>
     <col min="1" max="1" width="10.2857142857143" style="4" customWidth="1"/>
     <col min="2" max="2" width="14" style="5" customWidth="1"/>
-    <col min="5" max="5" width="11" customWidth="1"/>
-    <col min="6" max="6" width="12.4285714285714" customWidth="1"/>
+    <col min="4" max="4" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:6">
+    <row r="1" s="3" customFormat="1" spans="1:4">
       <c r="A1" s="6" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>15</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4">
       <c r="A2" s="8" t="s">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>0</v>
-      </c>
-      <c r="E2">
         <v>2</v>
       </c>
-      <c r="F2">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" s="8" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>0</v>
-      </c>
-      <c r="E3">
         <v>2</v>
       </c>
-      <c r="F3">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+    </row>
+    <row r="4" spans="1:4">
       <c r="A4" s="8" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D4">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="8" t="s">
+        <v>95</v>
+      </c>
+      <c r="B5" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5">
         <v>2</v>
       </c>
-      <c r="E4">
+      <c r="D5">
         <v>6</v>
       </c>
-      <c r="F4">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="8" t="s">
-        <v>102</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>2</v>
-      </c>
-      <c r="E5">
-        <v>6</v>
-      </c>
-      <c r="F5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" ht="24" spans="1:6">
+    </row>
+    <row r="6" ht="24" spans="1:4">
       <c r="A6" s="8" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>0</v>
-      </c>
-      <c r="E6">
         <v>2</v>
       </c>
-      <c r="F6">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" ht="24" spans="1:6">
+    </row>
+    <row r="7" ht="24" spans="1:4">
       <c r="A7" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7">
+        <v>2</v>
+      </c>
+      <c r="D7">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" ht="24" spans="1:4">
+      <c r="A8" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8">
+        <v>2</v>
+      </c>
+      <c r="D8">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="B9" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9">
+        <v>1</v>
+      </c>
+      <c r="D9">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" ht="24" spans="1:4">
+      <c r="A10" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="B10" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C10">
+        <v>2</v>
+      </c>
+      <c r="D10">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" ht="24" spans="1:4">
+      <c r="A11" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="B11" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C11">
+        <v>2</v>
+      </c>
+      <c r="D11">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12" ht="24" spans="1:4">
+      <c r="A12" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="B12" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C12">
+        <v>2</v>
+      </c>
+      <c r="D12">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" ht="24" spans="1:4">
+      <c r="A13" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="C13">
+        <v>2</v>
+      </c>
+      <c r="D13">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4">
+      <c r="A14" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7">
-        <v>2</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" ht="24" spans="1:6">
-      <c r="A8" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>2</v>
-      </c>
-      <c r="E8">
-        <v>6</v>
-      </c>
-      <c r="F8">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="B9" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>2</v>
-      </c>
-      <c r="F9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" ht="24" spans="1:6">
-      <c r="A10" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="B10" s="9" t="s">
+      <c r="B14" s="9" t="s">
         <v>49</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10">
-        <v>2</v>
-      </c>
-      <c r="E10">
-        <v>6</v>
-      </c>
-      <c r="F10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" ht="24" spans="1:6">
-      <c r="A11" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>2</v>
-      </c>
-      <c r="E11">
-        <v>6</v>
-      </c>
-      <c r="F11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" ht="24" spans="1:6">
-      <c r="A12" s="8" t="s">
-        <v>109</v>
-      </c>
-      <c r="B12" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C12">
-        <v>0</v>
-      </c>
-      <c r="D12">
-        <v>2</v>
-      </c>
-      <c r="E12">
-        <v>6</v>
-      </c>
-      <c r="F12">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" ht="24" spans="1:6">
-      <c r="A13" s="8" t="s">
-        <v>110</v>
-      </c>
-      <c r="B13" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="C13">
-        <v>0</v>
-      </c>
-      <c r="D13">
-        <v>2</v>
-      </c>
-      <c r="E13">
-        <v>6</v>
-      </c>
-      <c r="F13">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="8" t="s">
-        <v>111</v>
-      </c>
-      <c r="B14" s="9" t="s">
-        <v>54</v>
       </c>
       <c r="C14">
         <v>0</v>
       </c>
       <c r="D14">
-        <v>0</v>
-      </c>
-      <c r="E14">
         <v>2</v>
       </c>
-      <c r="F14">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" ht="24" spans="1:6">
+    </row>
+    <row r="15" ht="24" spans="1:4">
       <c r="A15" s="8" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
       <c r="D15">
-        <v>0</v>
-      </c>
-      <c r="E15">
         <v>2</v>
       </c>
-      <c r="F15">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6">
+    </row>
+    <row r="16" spans="1:4">
       <c r="A16" s="8" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="C16">
         <v>0</v>
       </c>
       <c r="D16">
-        <v>0</v>
-      </c>
-      <c r="E16">
         <v>2</v>
       </c>
-      <c r="F16">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" ht="24" spans="1:6">
+    </row>
+    <row r="17" ht="24" spans="1:4">
       <c r="A17" s="8" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="C17">
         <v>0</v>
       </c>
       <c r="D17">
-        <v>0</v>
-      </c>
-      <c r="E17">
         <v>2</v>
       </c>
-      <c r="F17">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" ht="24" spans="1:6">
+    </row>
+    <row r="18" ht="24" spans="1:4">
       <c r="A18" s="8" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C18">
         <v>0</v>
       </c>
       <c r="D18">
-        <v>0</v>
-      </c>
-      <c r="E18">
         <v>2</v>
       </c>
-      <c r="F18">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="19" ht="24" spans="1:6">
+    </row>
+    <row r="19" ht="24" spans="1:4">
       <c r="A19" s="8" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="C19">
         <v>0</v>
       </c>
       <c r="D19">
-        <v>0</v>
-      </c>
-      <c r="E19">
         <v>2</v>
       </c>
-      <c r="F19">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="20" ht="36" spans="1:6">
+    </row>
+    <row r="20" ht="36" spans="1:4">
       <c r="A20" s="8" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C20">
         <v>0</v>
       </c>
       <c r="D20">
-        <v>0</v>
-      </c>
-      <c r="E20">
         <v>2</v>
       </c>
-      <c r="F20">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6">
+    </row>
+    <row r="21" spans="1:4">
       <c r="A21" s="8" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C21">
         <v>0</v>
       </c>
       <c r="D21">
-        <v>0</v>
-      </c>
-      <c r="E21">
         <v>2</v>
       </c>
-      <c r="F21">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" ht="24" spans="1:6">
+    </row>
+    <row r="22" ht="24" spans="1:4">
       <c r="A22" s="8" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C22">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22">
-        <v>1</v>
-      </c>
-      <c r="E22">
         <v>2</v>
       </c>
-      <c r="F22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" ht="24" spans="1:6">
+    </row>
+    <row r="23" ht="24" spans="1:4">
       <c r="A23" s="8" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="C23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D23">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" ht="24" spans="1:4">
+      <c r="A24" s="8" t="s">
+        <v>114</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24">
         <v>2</v>
       </c>
-      <c r="E23">
+      <c r="D24">
         <v>6</v>
       </c>
-      <c r="F23">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="24" ht="24" spans="1:6">
-      <c r="A24" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="B24" s="9" t="s">
-        <v>91</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="E24">
-        <v>6</v>
-      </c>
-      <c r="F24">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" ht="24" spans="1:6">
+    </row>
+    <row r="25" ht="24" spans="1:4">
       <c r="A25" s="8" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="C25">
         <v>0</v>
       </c>
       <c r="D25">
-        <v>0</v>
-      </c>
-      <c r="E25">
         <v>2</v>
-      </c>
-      <c r="F25">
-        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -3579,90 +2844,62 @@
   <dimension ref="A1:A11"/>
   <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="10.8571428571429" style="2" customWidth="1"/>
+    <col min="1" max="1" width="10.8571428571429" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="2" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" s="1" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" s="1" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" s="1" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" s="2" t="s">
+    <row r="9" spans="1:1">
+      <c r="A9" s="1" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="3" spans="1:1">
-      <c r="A3" s="2" t="s">
+    <row r="10" spans="1:1">
+      <c r="A10" s="1" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="4" spans="1:1">
-      <c r="A4" s="2" t="s">
+    <row r="11" spans="1:1">
+      <c r="A11" s="1" t="s">
         <v>126</v>
-      </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="2" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="7" spans="1:1">
-      <c r="A7" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1">
-      <c r="A8" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1">
-      <c r="A9" s="2" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1">
-      <c r="A10" s="2" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="11" spans="1:1">
-      <c r="A11" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultColWidth="9.14285714285714" defaultRowHeight="15" outlineLevelRow="1" outlineLevelCol="1"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>134</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1">
-        <v>2023</v>
-      </c>
-      <c r="B2" s="1">
-        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>